<commit_message>
Facility Data 추가, RequireResearch, RequireCoreLevel 컬럼 추가
</commit_message>
<xml_diff>
--- a/Assets/100_Data/XlsxFiles/Item_Data.xlsx
+++ b/Assets/100_Data/XlsxFiles/Item_Data.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="172">
   <si>
     <t>Id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -170,50 +170,22 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>UnitId</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>stone_miner1</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>stone_miner2</t>
-  </si>
-  <si>
-    <t>stone_miner3</t>
-  </si>
-  <si>
     <t>stone_processor1</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>stone_processor2</t>
-  </si>
-  <si>
-    <t>stone_processor3</t>
-  </si>
-  <si>
     <t>돌 채굴 시설 Lv.1</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>돌 채굴 시설 Lv.2</t>
-  </si>
-  <si>
-    <t>돌 채굴 시설 Lv.3</t>
-  </si>
-  <si>
     <t>돌 가공 시설 Lv.1</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>돌 가공 시설 Lv.2</t>
-  </si>
-  <si>
-    <t>돌 가공 시설 Lv.3</t>
-  </si>
-  <si>
     <t>Facility</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -314,14 +286,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>옵시디언 광물</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>옵시디언 자재</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>텅스텐 광물</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -422,6 +386,251 @@
   </si>
   <si>
     <t>철 가공 시설 Lv.3</t>
+  </si>
+  <si>
+    <t>흑요석 광물</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>흑요석 자재</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>lab6</t>
+  </si>
+  <si>
+    <t>연구소 Lv.6</t>
+  </si>
+  <si>
+    <t>lab7</t>
+  </si>
+  <si>
+    <t>연구소 Lv.7</t>
+  </si>
+  <si>
+    <t>engineMerger6</t>
+  </si>
+  <si>
+    <t>엔진 합성기 Lv.6</t>
+  </si>
+  <si>
+    <t>engineMerger7</t>
+  </si>
+  <si>
+    <t>엔진 합성기 Lv.7</t>
+  </si>
+  <si>
+    <t>자원 합성기 Lv.1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>resource_merger2</t>
+  </si>
+  <si>
+    <t>자원 합성기 Lv.2</t>
+  </si>
+  <si>
+    <t>resource_merger3</t>
+  </si>
+  <si>
+    <t>자원 합성기 Lv.3</t>
+  </si>
+  <si>
+    <t>resource_merger4</t>
+  </si>
+  <si>
+    <t>자원 합성기 Lv.4</t>
+  </si>
+  <si>
+    <t>resource_merger5</t>
+  </si>
+  <si>
+    <t>자원 합성기 Lv.5</t>
+  </si>
+  <si>
+    <t>resource_merger6</t>
+  </si>
+  <si>
+    <t>자원 합성기 Lv.6</t>
+  </si>
+  <si>
+    <t>resource_merger7</t>
+  </si>
+  <si>
+    <t>자원 합성기 Lv.7</t>
+  </si>
+  <si>
+    <t>resource_merger1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>gold_miner2</t>
+  </si>
+  <si>
+    <t>금 채굴 시설 Lv.2</t>
+  </si>
+  <si>
+    <t>gold_miner3</t>
+  </si>
+  <si>
+    <t>금 채굴 시설 Lv.3</t>
+  </si>
+  <si>
+    <t>금 가공 시설 Lv.1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>gold_processor2</t>
+  </si>
+  <si>
+    <t>금 가공 시설 Lv.2</t>
+  </si>
+  <si>
+    <t>gold_processor3</t>
+  </si>
+  <si>
+    <t>금 가공 시설 Lv.3</t>
+  </si>
+  <si>
+    <t>obsidian_miner1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>obsidian_miner2</t>
+  </si>
+  <si>
+    <t>흑요석 채굴 시설 Lv.2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>obsidian_miner3</t>
+  </si>
+  <si>
+    <t>흑요석 채굴 시설 Lv.3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>obsidian_processor1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>흑요석 가공 시설 Lv.1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>obsidian_processor2</t>
+  </si>
+  <si>
+    <t>흑요석 가공 시설 Lv.2</t>
+  </si>
+  <si>
+    <t>obsidian_processor3</t>
+  </si>
+  <si>
+    <t>흑요석 가공 시설 Lv.3</t>
+  </si>
+  <si>
+    <t>tunstein_miner2</t>
+  </si>
+  <si>
+    <t>텅스텐 채굴 시설 Lv.2</t>
+  </si>
+  <si>
+    <t>tunstein_miner3</t>
+  </si>
+  <si>
+    <t>텅스텐 채굴 시설 Lv.3</t>
+  </si>
+  <si>
+    <t>tunstein_processor1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>tunstein_processor2</t>
+  </si>
+  <si>
+    <t>텅스텐 가공 시설 Lv.2</t>
+  </si>
+  <si>
+    <t>tunstein_processor3</t>
+  </si>
+  <si>
+    <t>텅스텐 가공 시설 Lv.3</t>
+  </si>
+  <si>
+    <t>titanium_miner1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>titanium_miner2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>티타늄 채굴 시설 Lv.2</t>
+  </si>
+  <si>
+    <t>titanium_processor1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>titanium_processor2</t>
+  </si>
+  <si>
+    <t>티타늄 가공 시설 Lv.2</t>
+  </si>
+  <si>
+    <t>titanium_processor3</t>
+  </si>
+  <si>
+    <t>티타늄 가공 시설 Lv.3</t>
+  </si>
+  <si>
+    <t>흑요석 채굴 시설 Lv.1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>텅스텐 채굴 시설 Lv.1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>티타늄 채굴 시설 Lv.1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>티타늄 채굴 시설 Lv.3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>티타늄 가공 시설 Lv.1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>gold_miner1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>금 채굴 시설 Lv.1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>gold_processor1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>tunstein_miner1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>텅스텐 가공 시설 Lv.1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>titanium_miner3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>EntityId</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -590,14 +799,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="표1" displayName="표1" ref="A1:F49" totalsRowShown="0">
-  <autoFilter ref="A1:F49"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="표1" displayName="표1" ref="A1:F80" totalsRowShown="0">
+  <autoFilter ref="A1:F80"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="4" name="Name"/>
     <tableColumn id="2" name="DisplayName"/>
     <tableColumn id="5" name="ItemType"/>
-    <tableColumn id="6" name="UnitId"/>
+    <tableColumn id="6" name="EntityId"/>
     <tableColumn id="3" name="ItemIcon"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -867,7 +1076,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F80"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="17.875" customWidth="1"/>
@@ -890,7 +1099,7 @@
         <v>20</v>
       </c>
       <c r="E1" t="s">
-        <v>38</v>
+        <v>171</v>
       </c>
       <c r="F1" t="s">
         <v>2</v>
@@ -1037,10 +1246,10 @@
         <v>1009</v>
       </c>
       <c r="B10" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="C10" t="s">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="D10" t="s">
         <v>21</v>
@@ -1054,10 +1263,10 @@
         <v>1010</v>
       </c>
       <c r="B11" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="C11" t="s">
-        <v>81</v>
+        <v>100</v>
       </c>
       <c r="D11" t="s">
         <v>21</v>
@@ -1071,10 +1280,10 @@
         <v>1011</v>
       </c>
       <c r="B12" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="C12" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="D12" t="s">
         <v>21</v>
@@ -1088,10 +1297,10 @@
         <v>1012</v>
       </c>
       <c r="B13" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="C13" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="D13" t="s">
         <v>21</v>
@@ -1105,10 +1314,10 @@
         <v>1013</v>
       </c>
       <c r="B14" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="C14" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="D14" t="s">
         <v>21</v>
@@ -1122,10 +1331,10 @@
         <v>1014</v>
       </c>
       <c r="B15" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="C15" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="D15" t="s">
         <v>21</v>
@@ -1259,13 +1468,13 @@
         <v>1201</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="E22" s="5">
         <v>101011</v>
@@ -1276,99 +1485,99 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
-        <v>1202</v>
+        <v>1204</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="E23" s="2">
-        <v>101012</v>
+        <v>101021</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="4">
-        <v>1203</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="E24" s="5">
-        <v>101013</v>
-      </c>
-      <c r="F24" s="6" t="s">
+      <c r="A24" s="1">
+        <v>1207</v>
+      </c>
+      <c r="B24" t="s">
+        <v>75</v>
+      </c>
+      <c r="C24" t="s">
+        <v>76</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E24">
+        <v>102011</v>
+      </c>
+      <c r="F24" s="3" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
-        <v>1204</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>48</v>
+        <v>1208</v>
+      </c>
+      <c r="B25" t="s">
+        <v>77</v>
+      </c>
+      <c r="C25" t="s">
+        <v>78</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E25" s="2">
-        <v>101021</v>
+        <v>42</v>
+      </c>
+      <c r="E25">
+        <v>102012</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="4">
-        <v>1205</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="E26" s="5">
-        <v>101022</v>
-      </c>
-      <c r="F26" s="6" t="s">
+      <c r="A26" s="1">
+        <v>1209</v>
+      </c>
+      <c r="B26" t="s">
+        <v>79</v>
+      </c>
+      <c r="C26" t="s">
+        <v>80</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E26">
+        <v>102013</v>
+      </c>
+      <c r="F26" s="3" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
-        <v>1206</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>50</v>
+        <v>1210</v>
+      </c>
+      <c r="B27" t="s">
+        <v>81</v>
+      </c>
+      <c r="C27" t="s">
+        <v>82</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E27" s="2">
-        <v>101023</v>
+        <v>42</v>
+      </c>
+      <c r="E27">
+        <v>102021</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>37</v>
@@ -1376,19 +1585,19 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
-        <v>1207</v>
+        <v>1211</v>
       </c>
       <c r="B28" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C28" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="E28">
-        <v>102011</v>
+        <v>102022</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>37</v>
@@ -1396,19 +1605,19 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
-        <v>1208</v>
+        <v>1212</v>
       </c>
       <c r="B29" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C29" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="E29">
-        <v>102012</v>
+        <v>102023</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>37</v>
@@ -1416,19 +1625,19 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
-        <v>1209</v>
+        <v>1213</v>
       </c>
       <c r="B30" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C30" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="E30">
-        <v>102013</v>
+        <v>103011</v>
       </c>
       <c r="F30" s="3" t="s">
         <v>37</v>
@@ -1436,19 +1645,19 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
-        <v>1210</v>
+        <v>1214</v>
       </c>
       <c r="B31" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C31" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="E31">
-        <v>102021</v>
+        <v>103012</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>37</v>
@@ -1456,19 +1665,19 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
-        <v>1211</v>
+        <v>1215</v>
       </c>
       <c r="B32" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C32" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="E32">
-        <v>102022</v>
+        <v>103013</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>37</v>
@@ -1476,19 +1685,19 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
-        <v>1212</v>
+        <v>1216</v>
       </c>
       <c r="B33" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C33" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="E33">
-        <v>102023</v>
+        <v>103021</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>37</v>
@@ -1496,19 +1705,19 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
-        <v>1213</v>
+        <v>1217</v>
       </c>
       <c r="B34" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C34" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="E34">
-        <v>103011</v>
+        <v>103022</v>
       </c>
       <c r="F34" s="3" t="s">
         <v>37</v>
@@ -1516,19 +1725,19 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
-        <v>1214</v>
+        <v>1218</v>
       </c>
       <c r="B35" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C35" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="E35">
-        <v>103012</v>
+        <v>103023</v>
       </c>
       <c r="F35" s="3" t="s">
         <v>37</v>
@@ -1536,19 +1745,19 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
-        <v>1215</v>
+        <v>1219</v>
       </c>
       <c r="B36" t="s">
-        <v>102</v>
+        <v>165</v>
       </c>
       <c r="C36" t="s">
-        <v>103</v>
+        <v>166</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="E36">
-        <v>103013</v>
+        <v>104011</v>
       </c>
       <c r="F36" s="3" t="s">
         <v>37</v>
@@ -1556,19 +1765,19 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
-        <v>1216</v>
+        <v>1220</v>
       </c>
       <c r="B37" t="s">
-        <v>104</v>
+        <v>123</v>
       </c>
       <c r="C37" t="s">
-        <v>105</v>
+        <v>124</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="E37">
-        <v>103021</v>
+        <v>104012</v>
       </c>
       <c r="F37" s="3" t="s">
         <v>37</v>
@@ -1576,19 +1785,19 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="1">
-        <v>1217</v>
+        <v>1221</v>
       </c>
       <c r="B38" t="s">
-        <v>106</v>
+        <v>125</v>
       </c>
       <c r="C38" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="E38">
-        <v>103022</v>
+        <v>104013</v>
       </c>
       <c r="F38" s="3" t="s">
         <v>37</v>
@@ -1596,222 +1805,821 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="1">
-        <v>1218</v>
+        <v>1222</v>
       </c>
       <c r="B39" t="s">
-        <v>108</v>
+        <v>167</v>
       </c>
       <c r="C39" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="E39">
-        <v>103023</v>
+        <v>104021</v>
       </c>
       <c r="F39" s="3" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="4">
-        <v>1301</v>
-      </c>
-      <c r="B40" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="C40" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="D40" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="E40" s="5">
-        <v>110001</v>
-      </c>
-      <c r="F40" s="6" t="s">
-        <v>72</v>
+      <c r="A40" s="1">
+        <v>1223</v>
+      </c>
+      <c r="B40" t="s">
+        <v>128</v>
+      </c>
+      <c r="C40" t="s">
+        <v>129</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E40">
+        <v>104022</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="1">
-        <v>1302</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>54</v>
+        <v>1224</v>
+      </c>
+      <c r="B41" t="s">
+        <v>130</v>
+      </c>
+      <c r="C41" t="s">
+        <v>131</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E41" s="2">
-        <v>110002</v>
+        <v>42</v>
+      </c>
+      <c r="E41">
+        <v>104023</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>72</v>
+        <v>37</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="4">
-        <v>1303</v>
-      </c>
-      <c r="B42" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="C42" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D42" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="E42" s="5">
-        <v>110003</v>
-      </c>
-      <c r="F42" s="6" t="s">
-        <v>72</v>
+      <c r="A42" s="1">
+        <v>1225</v>
+      </c>
+      <c r="B42" t="s">
+        <v>132</v>
+      </c>
+      <c r="C42" t="s">
+        <v>160</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E42">
+        <v>105011</v>
+      </c>
+      <c r="F42" s="3" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="1">
-        <v>1304</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>56</v>
+        <v>1226</v>
+      </c>
+      <c r="B43" t="s">
+        <v>133</v>
+      </c>
+      <c r="C43" t="s">
+        <v>134</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E43" s="2">
-        <v>110004</v>
+        <v>42</v>
+      </c>
+      <c r="E43">
+        <v>105012</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>72</v>
+        <v>37</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A44" s="4">
-        <v>1305</v>
-      </c>
-      <c r="B44" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="C44" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="D44" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="E44" s="5">
-        <v>110005</v>
-      </c>
-      <c r="F44" s="6" t="s">
-        <v>72</v>
+      <c r="A44" s="1">
+        <v>1227</v>
+      </c>
+      <c r="B44" t="s">
+        <v>135</v>
+      </c>
+      <c r="C44" t="s">
+        <v>136</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E44">
+        <v>105013</v>
+      </c>
+      <c r="F44" s="3" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" s="1">
-        <v>1401</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>63</v>
+        <v>1228</v>
+      </c>
+      <c r="B45" t="s">
+        <v>137</v>
+      </c>
+      <c r="C45" t="s">
+        <v>138</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E45" s="2">
-        <v>111001</v>
+        <v>42</v>
+      </c>
+      <c r="E45">
+        <v>105021</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>73</v>
+        <v>37</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A46" s="4">
-        <v>1402</v>
-      </c>
-      <c r="B46" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="C46" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="D46" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="E46" s="5">
-        <v>111002</v>
-      </c>
-      <c r="F46" s="6" t="s">
-        <v>73</v>
+      <c r="A46" s="1">
+        <v>1229</v>
+      </c>
+      <c r="B46" t="s">
+        <v>139</v>
+      </c>
+      <c r="C46" t="s">
+        <v>140</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E46">
+        <v>105022</v>
+      </c>
+      <c r="F46" s="3" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="1">
+        <v>1230</v>
+      </c>
+      <c r="B47" t="s">
+        <v>141</v>
+      </c>
+      <c r="C47" t="s">
+        <v>142</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E47">
+        <v>105023</v>
+      </c>
+      <c r="F47" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A48" s="1">
+        <v>1231</v>
+      </c>
+      <c r="B48" t="s">
+        <v>168</v>
+      </c>
+      <c r="C48" t="s">
+        <v>161</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E48">
+        <v>106011</v>
+      </c>
+      <c r="F48" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A49" s="1">
+        <v>1232</v>
+      </c>
+      <c r="B49" t="s">
+        <v>143</v>
+      </c>
+      <c r="C49" t="s">
+        <v>144</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E49">
+        <v>106012</v>
+      </c>
+      <c r="F49" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A50" s="1">
+        <v>1233</v>
+      </c>
+      <c r="B50" t="s">
+        <v>145</v>
+      </c>
+      <c r="C50" t="s">
+        <v>146</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E50">
+        <v>106013</v>
+      </c>
+      <c r="F50" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A51" s="1">
+        <v>1234</v>
+      </c>
+      <c r="B51" t="s">
+        <v>147</v>
+      </c>
+      <c r="C51" t="s">
+        <v>169</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E51">
+        <v>106021</v>
+      </c>
+      <c r="F51" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A52" s="1">
+        <v>1235</v>
+      </c>
+      <c r="B52" t="s">
+        <v>148</v>
+      </c>
+      <c r="C52" t="s">
+        <v>149</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E52">
+        <v>106022</v>
+      </c>
+      <c r="F52" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A53" s="1">
+        <v>1236</v>
+      </c>
+      <c r="B53" t="s">
+        <v>150</v>
+      </c>
+      <c r="C53" t="s">
+        <v>151</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E53">
+        <v>106023</v>
+      </c>
+      <c r="F53" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A54" s="1">
+        <v>1237</v>
+      </c>
+      <c r="B54" t="s">
+        <v>152</v>
+      </c>
+      <c r="C54" t="s">
+        <v>162</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E54">
+        <v>107011</v>
+      </c>
+      <c r="F54" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A55" s="1">
+        <v>1238</v>
+      </c>
+      <c r="B55" t="s">
+        <v>153</v>
+      </c>
+      <c r="C55" t="s">
+        <v>154</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E55">
+        <v>107012</v>
+      </c>
+      <c r="F55" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A56" s="1">
+        <v>1239</v>
+      </c>
+      <c r="B56" t="s">
+        <v>170</v>
+      </c>
+      <c r="C56" t="s">
+        <v>163</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E56">
+        <v>107013</v>
+      </c>
+      <c r="F56" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A57" s="1">
+        <v>1240</v>
+      </c>
+      <c r="B57" t="s">
+        <v>155</v>
+      </c>
+      <c r="C57" t="s">
+        <v>164</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E57">
+        <v>107021</v>
+      </c>
+      <c r="F57" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A58" s="1">
+        <v>1241</v>
+      </c>
+      <c r="B58" t="s">
+        <v>156</v>
+      </c>
+      <c r="C58" t="s">
+        <v>157</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E58">
+        <v>107022</v>
+      </c>
+      <c r="F58" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A59" s="1">
+        <v>1242</v>
+      </c>
+      <c r="B59" t="s">
+        <v>158</v>
+      </c>
+      <c r="C59" t="s">
+        <v>159</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E59">
+        <v>107023</v>
+      </c>
+      <c r="F59" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A60" s="4">
+        <v>1301</v>
+      </c>
+      <c r="B60" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C60" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D60" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E60" s="5">
+        <v>110001</v>
+      </c>
+      <c r="F60" s="6" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A61" s="1">
+        <v>1302</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E61" s="2">
+        <v>110002</v>
+      </c>
+      <c r="F61" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A62" s="4">
+        <v>1303</v>
+      </c>
+      <c r="B62" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C62" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D62" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E62" s="5">
+        <v>110003</v>
+      </c>
+      <c r="F62" s="6" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A63" s="1">
+        <v>1304</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E63" s="2">
+        <v>110004</v>
+      </c>
+      <c r="F63" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A64" s="4">
+        <v>1305</v>
+      </c>
+      <c r="B64" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C64" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D64" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E64" s="5">
+        <v>110005</v>
+      </c>
+      <c r="F64" s="6" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A65">
+        <v>1306</v>
+      </c>
+      <c r="B65" t="s">
+        <v>101</v>
+      </c>
+      <c r="C65" t="s">
+        <v>102</v>
+      </c>
+      <c r="D65" t="s">
+        <v>42</v>
+      </c>
+      <c r="E65">
+        <v>110006</v>
+      </c>
+      <c r="F65" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A66">
+        <v>1307</v>
+      </c>
+      <c r="B66" t="s">
+        <v>103</v>
+      </c>
+      <c r="C66" t="s">
+        <v>104</v>
+      </c>
+      <c r="D66" t="s">
+        <v>42</v>
+      </c>
+      <c r="E66">
+        <v>110007</v>
+      </c>
+      <c r="F66" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A67" s="1">
+        <v>1401</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E67" s="2">
+        <v>111001</v>
+      </c>
+      <c r="F67" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A68" s="4">
+        <v>1402</v>
+      </c>
+      <c r="B68" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C68" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D68" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E68" s="5">
+        <v>111002</v>
+      </c>
+      <c r="F68" s="6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A69" s="1">
         <v>1403</v>
       </c>
-      <c r="B47" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E47" s="2">
+      <c r="B69" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E69" s="2">
         <v>111003</v>
       </c>
-      <c r="F47" s="3" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48" s="4">
+      <c r="F69" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A70" s="4">
         <v>1404</v>
       </c>
-      <c r="B48" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="C48" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="D48" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="E48" s="5">
+      <c r="B70" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C70" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D70" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E70" s="5">
         <v>111004</v>
       </c>
-      <c r="F48" s="6" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="7">
+      <c r="F70" s="6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A71" s="7">
         <v>1405</v>
       </c>
-      <c r="B49" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="C49" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="D49" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="E49" s="8">
+      <c r="B71" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C71" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="D71" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E71" s="8">
         <v>111005</v>
       </c>
-      <c r="F49" s="9" t="s">
-        <v>73</v>
+      <c r="F71" s="9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A72" s="7">
+        <v>1406</v>
+      </c>
+      <c r="B72" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="C72" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="D72" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E72" s="8">
+        <v>111006</v>
+      </c>
+      <c r="F72" s="9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A73" s="7">
+        <v>1407</v>
+      </c>
+      <c r="B73" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="C73" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="D73" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E73" s="8">
+        <v>111007</v>
+      </c>
+      <c r="F73" s="9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A74">
+        <v>1501</v>
+      </c>
+      <c r="B74" t="s">
+        <v>122</v>
+      </c>
+      <c r="C74" t="s">
+        <v>109</v>
+      </c>
+      <c r="D74" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E74">
+        <v>113001</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A75">
+        <v>1502</v>
+      </c>
+      <c r="B75" t="s">
+        <v>110</v>
+      </c>
+      <c r="C75" t="s">
+        <v>111</v>
+      </c>
+      <c r="D75" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E75">
+        <v>113002</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A76">
+        <v>1503</v>
+      </c>
+      <c r="B76" t="s">
+        <v>112</v>
+      </c>
+      <c r="C76" t="s">
+        <v>113</v>
+      </c>
+      <c r="D76" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E76">
+        <v>113003</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A77">
+        <v>1504</v>
+      </c>
+      <c r="B77" t="s">
+        <v>114</v>
+      </c>
+      <c r="C77" t="s">
+        <v>115</v>
+      </c>
+      <c r="D77" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E77">
+        <v>113004</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A78">
+        <v>1505</v>
+      </c>
+      <c r="B78" t="s">
+        <v>116</v>
+      </c>
+      <c r="C78" t="s">
+        <v>117</v>
+      </c>
+      <c r="D78" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E78">
+        <v>113005</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A79">
+        <v>1506</v>
+      </c>
+      <c r="B79" t="s">
+        <v>118</v>
+      </c>
+      <c r="C79" t="s">
+        <v>119</v>
+      </c>
+      <c r="D79" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E79">
+        <v>113006</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A80">
+        <v>1507</v>
+      </c>
+      <c r="B80" t="s">
+        <v>120</v>
+      </c>
+      <c r="C80" t="s">
+        <v>121</v>
+      </c>
+      <c r="D80" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E80">
+        <v>113007</v>
       </c>
     </row>
   </sheetData>

</xml_diff>